<commit_message>
fw26: 50 design visualizations, panel migration, Etsy protocols and per-listing personalization
- images: 10 heroes + 40 gallery frames (nano_banana_2, 2k, count 1), tight hero crops as references,
  contact-sheet QA; 7 frames reshot (invented end-cap pattern, stone-textured enamel, hidden cells,
  wrong TI sign, two-piece seam). JPGs at public/artifact/fw26/Lxx/01..05.jpg. Not attached to any
  listing: the brief marks visualizations as internal mocks; owner decision pending.
- 0171 migration (not applied): 10 panel drafts, 282 variants, set seal fc12f228e903216ae566cbfcc204c0e2.
- listing-protocol: stick_pin (11316), shawl_pin (6066), ring_band (1232) from the live taxonomy.
- create-listing: listing_metadata.personalizationQuestions overrides the protocol question when well formed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155ChXCESvn4jMw6J2DsxxU
</commit_message>
<xml_diff>
--- a/docs/artifact-studio/fw26-trend-edit/exports/fw26-listings.xlsx
+++ b/docs/artifact-studio/fw26-trend-edit/exports/fw26-listings.xlsx
@@ -1135,7 +1135,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>On, required, max 16 characters. Pet name for the back (up to 10 characters) and DOG or CAT for the paw style. Example: BIBER / DOG. Add a year after the name if you are marking a life.</t>
+          <t>On, required, max 24 characters. Pet name for the back (up to 10 characters), then dog or cat for the paw. Example: Biber / dog. A year may follow.</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
         <is>
           <t>chain steps for 18 and 20 in: the reference listing's own base steps (same rule as L02, L05, L06). Panel prices of listing 4590337023 (Bauble) read 2026-10-17.
 grid rule (as the brief, same pattern as L04 and L06): as the brief: 3 x 3 x 4 = 36 variants. Paw Finish takes Etsy's third variation axis, so Metal Color cannot be a variation.
-personalization length: kept. A 10-character name plus ' / DOG' is 16, and the instructions invite a year as well: BIBER 2026 / DOG is 16, a 10-letter name with a year is 21 and would be cut off. Raise to 24 if Husam wants the year to fit every name.</t>
+personalization instructions: Pet name for the back (up to 10 characters), then dog or cat for the paw. Example: Biber / dog. A year may follow. (max 24). Etsy rejects personalization instructions over 120 characters and with more than one word starting with three capitals (developers.etsy.com personalization-migration, read 2026-10-17); the brief's text is 152 characters. Same meaning, shortened. Max characters raised so a 10-letter name plus a year fits (proposed at L09, covered by 'yes to all').</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>On, optional, max 40 characters. Two initials, almond bracelet first, then iris bracelet (example: H / C). Optional: a second length if the wrists differ (example: H 6.5 / C 7).</t>
+          <t>On, optional, max 40 characters. Two initials, almond bracelet first, then iris (e.g. H / C). Add a second length if wrists differ (e.g. H 6.5 / C 7).</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,8 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>category id: kept; resolved at push by the repo's chain_bracelet protocol (root Jewelry), the protocol the shop's earlier bracelet drafts were pushed with. lib/etsy/listing-protocol.ts chain_bracelet: taxonomyNames Chain &amp; Link Bracelets, Bracelets; taxonomyRoot Jewelry.</t>
+          <t>category id: kept; resolved at push by the repo's chain_bracelet protocol (root Jewelry), the protocol the shop's earlier bracelet drafts were pushed with. lib/etsy/listing-protocol.ts chain_bracelet: taxonomyNames Chain &amp; Link Bracelets, Bracelets; taxonomyRoot Jewelry.
+personalization instructions: Two initials, almond bracelet first, then iris (e.g. H / C). Add a second length if wrists differ (e.g. H 6.5 / C 7).. Etsy rejects personalization instructions over 120 characters and with more than one word starting with three capitals (developers.etsy.com personalization-migration, read 2026-10-17); the brief's text is 144 characters. Same meaning, shortened.</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3272,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>On, optional, max 5 characters. Up to 3 initials for the end cap, typed exactly as you want them cut (example: H.A. or HEA). Leave blank for no engraving.</t>
+          <t>On, optional, max 5 characters. Up to 3 initials for the end cap, typed exactly as you want them cut (e.g. H.A. or HEA). Blank means no engraving.</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3418,8 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>category: Accessories &gt; Pins &amp; Clips &gt; Hat Pins &amp; Stick Pins (taxonomy 11316). Live Etsy seller taxonomy read 2026-10-17 through ops/drafts-push?taxonomy=: no node contains 'lapel'; Pins &amp; Clips sits under Accessories with children Hat Pins &amp; Stick Pins (11316), Pins &amp; Pinback Buttons (41), Shawl Pins (6066), Brooches (1201). A stick pin with a clutch is a stick pin.</t>
+          <t>category: Accessories &gt; Pins &amp; Clips &gt; Hat Pins &amp; Stick Pins (taxonomy 11316). Live Etsy seller taxonomy read 2026-10-17 through ops/drafts-push?taxonomy=: no node contains 'lapel'; Pins &amp; Clips sits under Accessories with children Hat Pins &amp; Stick Pins (11316), Pins &amp; Pinback Buttons (41), Shawl Pins (6066), Brooches (1201). A stick pin with a clutch is a stick pin.
+personalization instructions: Up to 3 initials for the end cap, typed exactly as you want them cut (e.g. H.A. or HEA). Blank means no engraving.. Etsy rejects personalization instructions over 120 characters and with more than one word starting with three capitals (developers.etsy.com personalization-migration, read 2026-10-17); the brief's text is 122 characters. Same meaning, shortened.</t>
         </is>
       </c>
     </row>
@@ -4879,7 +4881,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>On, optional, max 8 characters. Up to 8 characters engraved on the back: initials, a year or a short word, typed exactly as you want them cut. Leave blank for a plain back.</t>
+          <t>On, optional, max 8 characters. Up to 8 characters for the back: initials, a year or a short word, typed as you want them cut. Blank: plain back.</t>
         </is>
       </c>
     </row>
@@ -5038,7 +5040,8 @@
       <c r="B24" s="4" t="inlineStr">
         <is>
           <t>chain steps for 18 and 20 in: the reference listing's own base steps (same rule as L02 and L05, approved). Panel prices of listing 4590337023 (Bauble) read 2026-10-17.
-grid rule (as the brief, same pattern as L04): as the brief: 3 x 3 x 4 = 36 variants. Sign takes Etsy's third variation axis, so Metal Color cannot be a variation; the brief routes white and rose through messages.</t>
+grid rule (as the brief, same pattern as L04): as the brief: 3 x 3 x 4 = 36 variants. Sign takes Etsy's third variation axis, so Metal Color cannot be a variation; the brief routes white and rose through messages.
+personalization instructions: Up to 8 characters for the back: initials, a year or a short word, typed as you want them cut. Blank: plain back.. Etsy rejects personalization instructions over 120 characters and with more than one word starting with three capitals (developers.etsy.com personalization-migration, read 2026-10-17); the brief's text is 140 characters. Same meaning, shortened.</t>
         </is>
       </c>
     </row>
@@ -5527,7 +5530,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>On, optional, max 40 characters. One initial per pendant, in order left to right (example: H / E / C). Optional: chain length per pendant, 16, 18 or 20 inches (example: H 16 / E 18 / C 18).</t>
+          <t>On, optional, max 40 characters. One initial per pendant, left to right (e.g. H / E / C). Add a chain length per pendant if needed (e.g. H 16 / E 18).</t>
         </is>
       </c>
     </row>
@@ -5685,7 +5688,8 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>overlap check: kept. The shop already sells a Solid 14K Gold Infinity Necklace (4579027067, wide open pendant) and two infinity bracelets. The Split Infinity differs as a cut, multi-piece matching set, and its title leads with 'Friendship Necklace Set', so it does not compete for the same search.</t>
+          <t>overlap check: kept. The shop already sells a Solid 14K Gold Infinity Necklace (4579027067, wide open pendant) and two infinity bracelets. The Split Infinity differs as a cut, multi-piece matching set, and its title leads with 'Friendship Necklace Set', so it does not compete for the same search.
+personalization instructions: One initial per pendant, left to right (e.g. H / E / C). Add a chain length per pendant if needed (e.g. H 16 / E 18).. Etsy rejects personalization instructions over 120 characters and with more than one word starting with three capitals (developers.etsy.com personalization-migration, read 2026-10-17); the brief's text is 156 characters. Same meaning, shortened.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fw26: visualizations become the listing images; panel loaded
- Owner chose the Higgsfield visualizations as listing images: every description gets the disclosure
  line, L06 and L09 no longer promise "photos", 0171 now inserts 5 listing_images per product.
- Applied to the panel through parts/: 10 products, 282 variants, 50 images; set seal
  fc12f228e903216ae566cbfcc204c0e2 and every per-listing variant, description and tag seal match;
  audit_log 10 / 282 / 50.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155ChXCESvn4jMw6J2DsxxU
</commit_message>
<xml_diff>
--- a/docs/artifact-studio/fw26-trend-edit/exports/fw26-listings.xlsx
+++ b/docs/artifact-studio/fw26-trend-edit/exports/fw26-listings.xlsx
@@ -1206,13 +1206,14 @@
       <c r="B18" s="4" t="inlineStr">
         <is>
           <t>A seal is the mark a thing leaves behind. The Paw Seal is a 10 mm solid gold disc with a paw pressed into its face as an intaglio, cut by hand below the surface the way a signet is cut, so it catches shadow rather than shine. The back carries your pet's name. Choose a plain gold paw, or have the intaglio filled with kiln-fired enamel in cobalt, cranberry or black.
-- The disc measures 10 mm across and 1.2 mm thick with a fixed bail; the paw is engraved by hand, and the two styles, dog and cat, are shown in the listing photos.
+- The disc measures 10 mm across and 1.2 mm thick with a fixed bail; the paw is engraved by hand, and the two styles, dog and cat, are shown side by side in the listing images.
 - Personalization: your pet's name on the back, up to 10 characters, and the choice of dog or cat paw. Add a year if you are marking a life.
 - Yellow gold as standard; message us for white or rose. Choose solid 10K, 14K or 18K with a 1.2 mm cable chain and spring ring clasp in 16, 18 or 20 inches. Message us for the bracelet version on a 6.5, 7 or 7.5 inch chain.
 - A personalized gift for a dog mom, a cat dad, a puppy's first Christmas, or in memory of a pet whose paw print is still on the car window.
 - Made to order at our bench in New Jersey in 5 to 7 business days, free US shipping, gift box included. Please check the spelling at checkout; engraved pieces are made specifically for you.
 - If you choose enamel, it is glass fused to gold and can chip from a hard knock; a soft cloth is all it needs. Gold itself does not tarnish.
-- A gift message can be added at checkout.</t>
+- A gift message can be added at checkout.
+- The product images are design visualizations of the finished piece, not photographs of a cast sample, and the multi-metal images are colour visualizations of the same design; the handmade piece may vary slightly.</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1531,8 @@
 - The enamel is fired by hand in a recessed cell with a polished gold rim, in the same cobalt as our Evil Eye collection, so the set stacks with it.
 - Made to order at our bench in New Jersey in 5 to 7 business days, free US shipping. The two bracelets arrive in separate gift boxes.
 - Please check the spelling at checkout; engraved pieces are made specifically for you.
-- Enamel is glass fused to gold and can chip from a hard knock. Take it off for the gym, the pool and the sink, and wipe it with a soft cloth. A gift message can be added at checkout.</t>
+- Enamel is glass fused to gold and can chip from a hard knock. Take it off for the gym, the pool and the sink, and wipe it with a soft cloth. A gift message can be added at checkout.
+- The product images are design visualizations of the finished piece, not photographs of a cast sample, and the multi-metal images are colour visualizations of the same design; the handmade piece may vary slightly.</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3339,8 @@
 - Wear it on a tuxedo lapel for a holiday party or an evening at the opera, or on a coat lapel on an ordinary Tuesday. It reads as heirloom jewelry, not as a novelty pin.
 - Made to order at our bench in New Jersey in 5 to 7 business days, then shipped free within the US with a solid gold clutch back and a gift box.
 - Gold does not tarnish. If the flutes collect dust, a soft brush and warm soapy water bring the shine back.
-- A gift message can be added at checkout. Please check the spelling at checkout; engraved pieces are made specifically for you.</t>
+- A gift message can be added at checkout. Please check the spelling at checkout; engraved pieces are made specifically for you.
+- The product images are design visualizations of the finished piece, not photographs of a cast sample, and the multi-metal images are colour visualizations of the same design; the handmade piece may vary slightly.</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3669,8 @@
 - Choose solid 10K, 14K or 18K gold in yellow, white or rose. Add a 1.2 mm cable chain in 16, 18 or 20 inches if you want to wear it as a pendant from day one.
 - It is made for the season of dressing up: a vintage style brooch for an evening coat, an opera night or a holiday table, and it stays in rotation long after.
 - Made to order at our bench in New Jersey in 3 to 5 business days, free US shipping, gift box included.
-- Garnet is hard enough for daily wear. Keep the piece away from knocks and clean it with a soft cloth. A gift message can be added at checkout.</t>
+- Garnet is hard enough for daily wear. Keep the piece away from knocks and clean it with a soft cloth. A gift message can be added at checkout.
+- The product images are design visualizations of the finished piece, not photographs of a cast sample, and the multi-metal images are colour visualizations of the same design; the handmade piece may vary slightly.</t>
         </is>
       </c>
     </row>
@@ -3983,7 +3987,8 @@
 - Wear it high on a capelet for an evening out, through a scarf on a coat, or as a sweater pin at the collarbone. It does the work of a brooch without the weight of one, and it is opera inspired in the oldest sense: dressing with intent.
 - Made to order at our bench in New Jersey in 3 to 5 business days, free US shipping, gift box included.
 - Gold does not tarnish. If the pin tip ever dulls on heavy wool, a few strokes on a fine emery board restore it. Avoid very loose, open weaves, where any pin can slip.
-- A gift message can be added at checkout.</t>
+- A gift message can be added at checkout.
+- The product images are design visualizations of the finished piece, not photographs of a cast sample, and the multi-metal images are colour visualizations of the same design; the handmade piece may vary slightly.</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4305,8 @@
 - Palette: Ur (lapis, red, white) for the original, or Festival (cobalt, cranberry, emerald, saffron and pink) when you want the full maximalist stack.
 - One Ur Band is a quiet accent of bold color. Two or three stacked with plain gold bands is the mood of this season, and it still works in July.
 - Made to order at our bench in New Jersey in 3 to 5 business days, free US shipping, gift box included.
-- Enamel is glass fused to gold and can chip from a hard knock. Take it off for the gym, the pool and the sink, and wipe it with a soft cloth. A gift message can be added at checkout.</t>
+- Enamel is glass fused to gold and can chip from a hard knock. Take it off for the gym, the pool and the sink, and wipe it with a soft cloth. A gift message can be added at checkout.
+- The product images are design visualizations of the finished piece, not photographs of a cast sample, and the multi-metal images are colour visualizations of the same design; the handmade piece may vary slightly.</t>
         </is>
       </c>
     </row>
@@ -4630,7 +4636,8 @@
 - It is a bold color piece that happens to be festive, which makes it an easy gift for a new home, a host, a friend who feeds everyone, or yourself, which is allowed.
 - Made to order at our bench in New Jersey in 3 to 5 business days, free US shipping, gift box included.
 - Enamel is glass fused to gold and can chip from a hard knock. Take it off for the gym, the pool and the sink, and wipe it with a soft cloth.
-- A gift message can be added at checkout.</t>
+- A gift message can be added at checkout.
+- The product images are design visualizations of the finished piece, not photographs of a cast sample, and the multi-metal images are colour visualizations of the same design; the handmade piece may vary slightly.</t>
         </is>
       </c>
     </row>
@@ -4953,12 +4960,13 @@
         <is>
           <t>Some of the first writing in the world was made by pressing a reed into wet clay. The marks became wedges, and the wedges became cuneiform. The Wedge pendant is a small bar of solid gold struck by hand with the same wedge shapes, one sign at a time, so every stroke is slightly deeper or lighter than the next. You choose the sign; the back is engraved with your initials or a date.
 - The bar measures 16 x 5 mm and 1 mm thick, rolled from solid gold sheet, annealed and hand stamped with three sizes of wedge punch. The surface is brushed, the edges softly rounded.
-- Four Sumerian signs to choose from: TI (life), SHA (heart), E (home) and AN (star, sky). The listing photos show each sign next to its meaning.
+- Four Sumerian signs to choose from: TI (life), SHA (heart), E (home) and AN (star, sky). The second image shows the four signs side by side, in this order.
 - Personalization: up to 8 characters engraved on the back, initials, a year or a short word, typed exactly as you want them cut.
 - Yellow gold as standard; message us for white or rose. Choose solid 10K, 14K or 18K with a 1.2 mm cable chain and spring ring clasp in 16, 18 or 20 inches.
 - Because each bar is struck by hand, spacing and depth vary a little from piece to piece. That variation is the point of the design, and it is why no two Wedges match.
 - Made to order at our bench in New Jersey in 5 to 7 business days, free US shipping, gift box included. Please check the spelling at checkout; engraved pieces are made specifically for you.
-- Gold does not tarnish; a soft cloth keeps the brushed finish even. A gift message can be added at checkout.</t>
+- Gold does not tarnish; a soft cloth keeps the brushed finish even. A gift message can be added at checkout.
+- The product images are design visualizations of the finished piece, not photographs of a cast sample, and the multi-metal images are colour visualizations of the same design; the handmade piece may vary slightly.</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5284,8 @@
 - Wear them alone, or as the second hoop in a stack. They sit well with velvet in December and with a T-shirt in June.
 - Made to order at our bench in New Jersey in 3 to 5 business days, free US shipping, gift box included.
 - Gold does not tarnish. Warm water with a drop of dish soap and a soft brush clears the texture of any residue.
-- A gift message can be added at checkout.</t>
+- A gift message can be added at checkout.
+- The product images are design visualizations of the finished piece, not photographs of a cast sample, and the multi-metal images are colour visualizations of the same design; the handmade piece may vary slightly.</t>
         </is>
       </c>
     </row>
@@ -5607,7 +5616,8 @@
 - The pieces are cast from one master and finished together as a set, so the break lines meet cleanly when the pendants are placed side by side.
 - Made to order at our bench in New Jersey in 5 to 7 business days, free US shipping. Each pendant arrives in its own gift box, so the set can be given in three places on the same night.
 - Please check the spelling at checkout; engraved pieces are made specifically for you.
-- Gold does not tarnish. A soft cloth keeps it bright. A gift message can be added at checkout.</t>
+- Gold does not tarnish. A soft cloth keeps it bright. A gift message can be added at checkout.
+- The product images are design visualizations of the finished piece, not photographs of a cast sample, and the multi-metal images are colour visualizations of the same design; the handmade piece may vary slightly.</t>
         </is>
       </c>
     </row>

</xml_diff>